<commit_message>
fix: center map tile switcher, fix Tabanan POI coordinates to render all 8 POIs in 500m catchment circle, add button spacing gap, and implement SHA-256 hashed password authentication
</commit_message>
<xml_diff>
--- a/BMN_Idle_Master_Backend.xlsx
+++ b/BMN_Idle_Master_Backend.xlsx
@@ -39592,7 +39592,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>password</t>
+          <t>password_hash</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -39624,7 +39624,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bmnidle2026</t>
+          <t>590909dbb0422b9a7e6cd906900ec3a6da7f6937ce1f52dc821f4d0ed8a99dd1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -39656,7 +39656,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>satker2026</t>
+          <t>7e765589b3df7c27c77ec54b5a661a800e8016fd78c9f8a909e415992e0e8a20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -39688,7 +39688,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>viewer2026</t>
+          <t>35cbe0aaf4e558ac53847cf7b057f4a3a86a427e08935bffdf81d7b4ed7cd9f3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>